<commit_message>
Release configure-gtm v10.2.0: verified native configuration and simpler execution
</commit_message>
<xml_diff>
--- a/tests/fixtures/tracking-plan-delivery/tracking-plan.xlsx
+++ b/tests/fixtures/tracking-plan-delivery/tracking-plan.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Event Matrix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Parameter Reference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="core_data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="view_item" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="begin_quote" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="__tracking_plan_model" sheetId="7" state="veryHidden" r:id="rId7"/>
-    <sheet name="__tracking_plan_projection" sheetId="8" state="veryHidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event Matrix" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter Reference" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="core_data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="view_item" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="begin_quote" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__tracking_plan_model" sheetId="7" state="veryHidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__tracking_plan_projection" sheetId="8" state="veryHidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Guide'!$A$15:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Event Matrix'!$A$4:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameter Reference'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameter Reference'!$A$4:$F$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'core_data'!$A$11:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'view_item'!$A$11:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'view_item'!$A$11:$G$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'begin_quote'!$A$11:$G$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,11 @@
       <name val="Consolas"/>
       <color rgb="00263238"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002F6F7E"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -186,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -206,9 +211,12 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -605,7 +613,13 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Approved — current-source checks passed</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -617,11 +631,11 @@
           <t>Example GA4 tracking plan</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="9" t="n"/>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -634,11 +648,11 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -651,11 +665,11 @@
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -668,11 +682,11 @@
           <t>Product discovery and quote request</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -685,11 +699,11 @@
           <t>to_be</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -702,47 +716,47 @@
           <t>en</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="8" t="n"/>
-    </row>
-    <row r="10" ht="28" customHeight="1">
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Analyst entry point</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Review journeys and events in Event Matrix.</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="28" customHeight="1">
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Developer entry point</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Open an event tab for the exact dataLayer specification.</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="28" customHeight="1">
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="9" t="n"/>
+    </row>
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>dataLayer convention</t>
@@ -754,11 +768,11 @@
 Clear event_data or ecommerce before replacing a previously populated object.</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="9" t="n"/>
     </row>
     <row r="13"/>
     <row r="14" ht="26" customHeight="1">
@@ -790,7 +804,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Product discovery</t>
@@ -812,7 +826,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Quote request</t>
@@ -836,11 +850,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A15:D17"/>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
+    <mergeCell ref="A3:G3"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B8:G8"/>
     <mergeCell ref="B4:G4"/>
@@ -899,7 +914,7 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>core_data</t>
         </is>
@@ -911,7 +926,7 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>view_item</t>
         </is>
@@ -923,7 +938,7 @@
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>begin_quote</t>
         </is>
@@ -955,7 +970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1013,7 +1028,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="94" customHeight="1">
+    <row r="5" ht="126" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>currency</t>
@@ -1137,7 +1152,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>SKU-123</t>
+          <t>Example: SKU-123</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1184,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Example window</t>
+          <t>Example: Example window</t>
         </is>
       </c>
     </row>
@@ -1201,11 +1216,11 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>120x100</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="66" customHeight="1">
+          <t>Example: 120x100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>items</t>
@@ -1233,7 +1248,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white"}]</t>
+          <t>See event-specific specifications: view_item</t>
         </is>
       </c>
     </row>
@@ -1301,104 +1316,168 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="126" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>project_type</t>
+          <t>price</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>item</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Identifies the normalized project selected for the quote request.</t>
+          <t>The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Use one of the exhaustive website project types.</t>
+          <t>Use the selected offer unit price excluding tax and shipping. This fictional supplied offer has no discount.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>window | door | shutter</t>
+          <t>Example: 129.9</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>project_type</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Identifies the normalized project selected for the quote request.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Use one of the exhaustive website project types.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>window | door | shutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Item quantity. If not set, quantity is set to 1.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Use 1 for the single displayed product unit.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Example: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>user</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>string or null</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>customer_12345</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="122" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Example: customer_12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>event</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value.</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Monetary value of the event’s items, excluding shipping and tax.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Set value to the sum of price * quantity for all items; exclude shipping and tax.</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>129.9</t>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Example: 129.9</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F18"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -1450,11 +1529,11 @@
           <t>core_data</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="9" t="n"/>
     </row>
     <row r="4" hidden="1" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1467,11 +1546,11 @@
           <t>dataLayer context</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="9" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1484,11 +1563,11 @@
           <t>Product discovery | Quote request</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1501,11 +1580,11 @@
           <t>Provides the reusable page and user context needed by subsequent measurement.</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1518,11 +1597,11 @@
           <t>Push on every full page load and SPA route change after page and user state are available, and refresh the same context after an authentication-state change.</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
     </row>
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1535,11 +1614,11 @@
           <t>all_pages | https://example.com/*</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
     <row r="9" hidden="1" ht="54" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1548,11 +1627,11 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
     </row>
     <row r="10"/>
     <row r="11" ht="34" customHeight="1">
@@ -1592,7 +1671,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="64" customHeight="1">
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>page_template</t>
@@ -1666,7 +1745,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="64" customHeight="1">
+    <row r="14" ht="171" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>user_id</t>
@@ -1679,7 +1758,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>string or null</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1694,7 +1773,8 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.</t>
+          <t>Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.
+Condition: Omit user_id before the first sign-in. Send the stable opaque account identifier as a string while signed in. After sign-out, send user_id as null to clear the GA4 User-ID setting.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1711,8 +1791,8 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="17" ht="156" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>window.dataLayer = window.dataLayer || [];
 window.dataLayer.push({
@@ -1752,7 +1832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1789,11 +1869,11 @@
           <t>view_item</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="9" t="n"/>
     </row>
     <row r="4" hidden="1" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1806,11 +1886,11 @@
           <t>official ecommerce</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="9" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1823,11 +1903,11 @@
           <t>Product discovery</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1840,11 +1920,11 @@
           <t>This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1857,11 +1937,11 @@
           <t>Push once after the primary product detail and selected default variant are rendered.</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
     </row>
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1874,11 +1954,11 @@
           <t>product_detail | https://example.com/products/{product} | Product detail</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
     <row r="9" hidden="1" ht="54" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1887,11 +1967,11 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
     </row>
     <row r="10"/>
     <row r="11" ht="34" customHeight="1">
@@ -1931,7 +2011,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="94" customHeight="1">
+    <row r="12" ht="126" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>currency</t>
@@ -1959,7 +2039,8 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Use the ISO 4217 currency code.</t>
+          <t>Use the ISO 4217 currency code.
+Condition: Required when value is sent.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1968,7 +2049,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="122" customHeight="1">
+    <row r="13" ht="64" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>value</t>
@@ -1991,7 +2072,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value.</t>
+          <t>Monetary value of the event’s items, excluding shipping and tax.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2005,7 +2086,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="66" customHeight="1">
+    <row r="14" ht="64" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>items</t>
@@ -2038,7 +2119,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white"}]</t>
+          <t>See the complete dataLayer example.</t>
         </is>
       </c>
     </row>
@@ -2190,16 +2271,90 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="19" ht="126" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>mandatory</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Use the selected offer unit price excluding tax and shipping. This fictional supplied offer has no discount.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>129.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>mandatory</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Item quantity. If not set, quantity is set to 1.</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Use 1 for the single displayed product unit.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>dataLayer specification</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="255" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="23" ht="291" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>window.dataLayer = window.dataLayer || [];
 window.dataLayer.push({"ecommerce": null});
@@ -2213,7 +2368,9 @@
         "item_id": "SKU-123",
         "item_name": "Example window",
         "item_variant": "120x100",
-        "item_color": "white"
+        "item_color": "white",
+        "price": 129.9,
+        "quantity": 1
       }
     ]
   }
@@ -2222,17 +2379,17 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A11:G18"/>
+  <autoFilter ref="A11:G20"/>
   <mergeCells count="11">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="B8:G8"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A23:G23"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="B6:G6"/>
   </mergeCells>
@@ -2283,11 +2440,11 @@
           <t>begin_quote</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n"/>
-      <c r="D3" s="7" t="n"/>
-      <c r="E3" s="7" t="n"/>
-      <c r="F3" s="7" t="n"/>
-      <c r="G3" s="8" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="9" t="n"/>
     </row>
     <row r="4" hidden="1" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -2300,11 +2457,11 @@
           <t>custom</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n"/>
-      <c r="D4" s="7" t="n"/>
-      <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="9" t="n"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -2317,11 +2474,11 @@
           <t>Quote request</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="n"/>
     </row>
     <row r="6" ht="54" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -2334,11 +2491,11 @@
           <t>Indicates that a visitor intentionally started the quote-request journey.</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="n"/>
     </row>
     <row r="7" ht="54" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -2351,11 +2508,11 @@
           <t>Push once when the visitor enters the first interactive quote step after selecting a quote call to action.</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="n"/>
     </row>
     <row r="8" ht="54" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -2368,11 +2525,11 @@
           <t>quote_form | https://example.com/request-a-quote | Quote form</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="n"/>
     </row>
     <row r="9" hidden="1" ht="54" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -2381,11 +2538,11 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="9" t="n"/>
     </row>
     <row r="10"/>
     <row r="11" ht="34" customHeight="1">
@@ -2462,7 +2619,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="64" customHeight="1">
+    <row r="13" ht="81" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>project_type</t>
@@ -2490,7 +2647,8 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Use one of the exhaustive website project types.</t>
+          <t>Use one of the exhaustive website project types.
+Condition: Send when the project type is known at journey start.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -2507,8 +2665,8 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="135" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="16" ht="141" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>window.dataLayer = window.dataLayer || [];
 window.dataLayer.push({"event_data": null});
@@ -2558,14 +2716,14 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>5.0.0</t>
+          <t>6.0.0</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"schema_version":"5.0.0","document":{"title":"Example GA4 tracking plan","version":"1.0","date":"2026-08-01","language":"en","scope":"Product discovery and quote request","target_state":"to_be"},"data_layer_convention":{"name":"Default web dataLayer","origin":"default","event_key":"event","wrappers":{"page":"page","event":"event_data","ecommerce":"ecommerce","user":"user"},"notes":"Clear event_data or ecommerce before replacing a previously populated object."},"journeys":[{"journey_id":"product_discovery","name":"Product discovery","scope":"Product detail pages","status":"observed","business_goal":"Understand qualified product interest.","urls":["https://example.com/products/{product}"]},{"journey_id":"quote_request","name":"Quote request","scope":"Quote form","status":"confirmed","business_goal":"Measure intentional quote starts and accepted leads.","urls":["https://example.com/request-a-quote"]}],"events":[{"event_name":"core_data","classification":"context","journey_ids":["product_discovery","quote_request"],"definition":"Provides the reusable page and user context needed by subsequent measurement.","trigger":"Push on every full page load and SPA route change after page and user state are available, and refresh the same context after an authentication-state change.","locations":[{"page_type":"all_pages","url_pattern":"https://example.com/*"}],"parameters":[{"name":"page_template","data_layer_path":"page.page_template","classification":"implementation","scope":"implementation","type":"string","requirement":"required","definition":"Identifies the stable functional template of the displayed page or route.","value_rule":"Use the normalized functional page template.","allowed_values":["home","product_detail","quote_form","confirmation"],"value_evidence_refs":["page_templates"],"example":"product_detail","source":"Application route metadata.","destination":"implementation_only","value_mode":"controlled_semantic","value_language":"en"},{"name":"login_status","data_layer_path":"user.login_status","classification":"custom","scope":"user","type":"string","requirement":"required","definition":"Indicates whether the current visitor is authenticated.","value_rule":"Use one of the exhaustive normalized states.","allowed_values":["logged_out","logged_in"],"value_evidence_refs":["login_statuses"],"example":"logged_in","source":"Authentication state.","destination":"ga4_user_property","custom_decision":{"business_need":"Compare journeys for authenticated and unauthenticated visitors.","official_candidate":"No prescribed event parameter represents reusable authentication state.","why_not_fit":"The value is persistent user context rather than the outcome of the official login event."},"value_mode":"controlled_semantic","value_language":"en"},{"name":"user_id","data_layer_path":"user.user_id","classification":"implementation","scope":"user","type":"string","requirement":"conditional","condition":"Send after authentication when a stable first-party User-ID is available; do not send before first sign-in and clear the GA4 setting with null after sign-out.","definition":"Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","value_rule":"Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.","example":"customer_12345","source":"Authenticated account state.","destination":"ga4_user_id","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/user-id","section":"Send user IDs","wording_origin":"faithful_translation","checked_date":"2026-08-01","official_text":"The user_id parameter is a configuration parameter, not a custom user property or standard event parameter."},"value_mode":"technical_identifier","value_evidence_refs":["user_ids"]}],"data_layer":{"push":{"page":{"page_template":"product_detail"},"user":{"login_status":"logged_in","user_id":"customer_12345"}}}},{"event_name":"view_item","classification":"official_ecommerce","journey_ids":["product_discovery"],"business_question":"Which products and selected variants attract consideration before later commerce actions?","definition":"This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","trigger":"Push once after the primary product detail and selected default variant are rendered.","locations":[{"page_type":"product_detail","url_pattern":"https://example.com/products/{product}","component":"Product detail"}],"parameters":[{"name":"currency","data_layer_path":"ecommerce.currency","classification":"official","scope":"event","type":"string","requirement":"conditional","condition":"Required when value is sent.","definition":"Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","value_rule":"Use the ISO 4217 currency code.","allowed_values":["EUR"],"value_evidence_refs":["currencies"],"example":"EUR","source":"Commerce currency configuration.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"exact","checked_date":"2026-08-01","official_text":"Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately."},"value_mode":"technical_identifier"},{"name":"value","data_layer_path":"ecommerce.value","classification":"official","scope":"event","type":"number","requirement":"optional","definition":"The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value.","value_rule":"Set value to the sum of price * quantity for all items; exclude shipping and tax.","example":129.9,"source":"Selected product offer.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value."},"value_mode":"numeric","value_evidence_refs":["item_values"]},{"name":"items","data_layer_path":"ecommerce.items","classification":"official","scope":"event","type":"array","requirement":"required","definition":"The items for the event.","value_rule":"Send one item object for the displayed product variant.","example":[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white"}],"source":"Selected product and variant data.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The items for the event."},"value_mode":"structured","value_evidence_refs":["item_arrays"]},{"name":"item_id","data_layer_path":"ecommerce.items[].item_id","classification":"official","scope":"item","type":"string","requirement":"required","definition":"The ID of the item. *One of item_id or item_name is required.","value_rule":"Use the stable SKU or product identifier.","example":"SKU-123","source":"Product catalog.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The ID of the item. *One of item_id or item_name is required."},"value_mode":"technical_identifier","value_evidence_refs":["item_ids"]},{"name":"item_name","data_layer_path":"ecommerce.items[].item_name","classification":"official","scope":"item","type":"string","requirement":"required","definition":"The name of the item. *One of item_id or item_name is required.","value_rule":"Use the stable catalog product name.","example":"Example window","source":"Product catalog.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The name of the item. *One of item_id or item_name is required."},"value_mode":"authoritative_raw","value_evidence_refs":["item_names"]},{"name":"item_variant","data_layer_path":"ecommerce.items[].item_variant","classification":"official","scope":"item","type":"string","requirement":"optional","definition":"The item variant or unique code or description for additional item details/options.","value_rule":"Use the primary normalized size or variant representation.","example":"120x100","source":"Selected variant.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The item variant or unique code or description for additional item details/options."},"value_mode":"authoritative_raw","value_evidence_refs":["item_variants"]},{"name":"item_color","data_layer_path":"ecommerce.items[].item_color","classification":"custom","scope":"item","type":"string","requirement":"optional","definition":"Identifies the normalized color selected for the item.","value_rule":"Use the normalized catalog color label.","allowed_values":["white","black","oak"],"value_evidence_refs":["item_colors"],"example":"white","source":"Selected variant color.","destination":"ga4_item_parameter","custom_decision":{"business_need":"Analyse color preference independently from size.","official_candidate":"item_variant","why_not_fit":"item_variant represents the primary size or variant; it cannot isolate color when both dimensions are selected."},"value_mode":"controlled_semantic","value_language":"en"}],"data_layer":{"clear":["ecommerce"],"push":{"event":"view_item","ecommerce":{"currency":"EUR","value":129.9,"items":[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white"}]}}},"official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item","wording_origin":"exact","checked_date":"2026-08-01","official_text":"This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed."},"measurement_opportunity_ids":["product_item_consideration"]},{"event_name":"begin_quote","classification":"custom","journey_ids":["quote_request"],"business_question":"How many visitors intentionally enter the quote journey, and for which project types?","definition":"Indicates that a visitor intentionally started the quote-request journey.","trigger":"Push once when the visitor enters the first interactive quote step after selecting a quote call to action.","locations":[{"page_type":"quote_form","url_pattern":"https://example.com/request-a-quote","component":"Quote form"}],"parameters":[{"name":"form_name","data_layer_path":"event_data.form_name","classification":"custom","scope":"event","type":"string","requirement":"required","definition":"Identifies the form whose journey was started.","value_rule":"Use the stable functional form name.","allowed_values":["quote_request"],"value_evidence_refs":["form_names"],"example":"quote_request","source":"Form configuration.","destination":"ga4_event_parameter","custom_decision":{"business_need":"Compare quote starts for reusable form implementations.","official_candidate":"No prescribed begin_quote parameter identifies the form.","why_not_fit":"A stable form identifier is required to analyse multiple quote entry points."},"value_mode":"controlled_semantic","value_language":"en"},{"name":"project_type","data_layer_path":"event_data.project_type","classification":"custom","scope":"event","type":"string","requirement":"conditional","condition":"Send when the project type is known at journey start.","definition":"Identifies the normalized project selected for the quote request.","value_rule":"Use one of the exhaustive website project types.","allowed_values":["window","door","shutter"],"value_evidence_refs":["project_types"],"example":"window","source":"Selected project option.","destination":"ga4_event_parameter","custom_decision":{"business_need":"Analyse quote starts by requested project.","official_candidate":"No official begin_quote parameter represents the requested project.","why_not_fit":"The project is a business-specific quote dimension."},"value_mode":"controlled_semantic","value_language":"en"}],"data_layer":{"clear":["event_data"],"push":{"event":"begin_quote","event_data":{"form_name":"quote_request","project_type":"window"}}},"custom_decision":{"business_need":"Measure intentional entry into a quote journey before a lead exists.","official_candidate":"form_start","why_not_fit":"The business requires a quote-specific funnel start across interfaces that do not all expose a standard form start."},"measurement_opportunity_ids":["quote_intentional_start"]}]}</t>
+          <t>{"schema_version":"6.0.0","document":{"title":"Example GA4 tracking plan","version":"1.0","date":"2026-08-01","language":"en","scope":"Product discovery and quote request","target_state":"to_be"},"data_layer_convention":{"name":"Default web dataLayer","origin":"default","event_key":"event","wrappers":{"page":"page","event":"event_data","ecommerce":"ecommerce","user":"user"},"notes":"Clear event_data or ecommerce before replacing a previously populated object."},"journeys":[{"journey_id":"product_discovery","name":"Product discovery","scope":"Product detail pages","status":"observed","business_goal":"Understand qualified product interest.","urls":["https://example.com/products/{product}"]},{"journey_id":"quote_request","name":"Quote request","scope":"Quote form","status":"confirmed","business_goal":"Measure intentional quote starts and accepted leads.","urls":["https://example.com/request-a-quote"]}],"events":[{"event_name":"core_data","classification":"context","journey_ids":["product_discovery","quote_request"],"definition":"Provides the reusable page and user context needed by subsequent measurement.","trigger":"Push on every full page load and SPA route change after page and user state are available, and refresh the same context after an authentication-state change.","locations":[{"page_type":"all_pages","url_pattern":"https://example.com/*"}],"parameters":[{"name":"page_template","data_layer_path":"page.page_template","classification":"implementation","scope":"implementation","type":"string","requirement":"required","definition":"Identifies the stable functional template of the displayed page or route.","value_rule":"Use the normalized functional page template.","allowed_values":["home","product_detail","quote_form","confirmation"],"value_evidence_refs":["page_templates"],"example":"product_detail","source":"Application route metadata.","destination":"implementation_only","value_mode":"controlled_semantic","value_language":"en"},{"name":"login_status","data_layer_path":"user.login_status","classification":"custom","scope":"user","type":"string","requirement":"required","definition":"Indicates whether the current visitor is authenticated.","value_rule":"Use one of the exhaustive normalized states.","allowed_values":["logged_out","logged_in"],"value_evidence_refs":["login_statuses"],"example":"logged_in","source":"Authentication state.","destination":"ga4_user_property","custom_decision":{"business_need":"Compare journeys for authenticated and unauthenticated visitors.","official_candidate":"No prescribed event parameter represents reusable authentication state.","why_not_fit":"The value is persistent user context rather than the outcome of the official login event."},"value_mode":"controlled_semantic","value_language":"en"},{"name":"user_id","data_layer_path":"user.user_id","classification":"implementation","scope":"user","type":"string","requirement":"conditional","nullable":true,"condition":"Omit user_id before the first sign-in. Send the stable opaque account identifier as a string while signed in. After sign-out, send user_id as null to clear the GA4 User-ID setting.","definition":"Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","value_rule":"Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.","example":"customer_12345","source":"Authenticated account state.","destination":"ga4_user_id","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/user-id","section":"Send user IDs","wording_origin":"faithful_adaptation","checked_date":"2026-08-01","official_text":"The user_id parameter is a configuration parameter, not a custom user property or standard event parameter."},"value_mode":"technical_identifier","value_evidence_refs":["user_ids"]}],"data_layer":{"push":{"page":{"page_template":"product_detail"},"user":{"login_status":"logged_in","user_id":"customer_12345"}}}},{"event_name":"view_item","classification":"official_ecommerce","journey_ids":["product_discovery"],"business_question":"Which products and selected variants attract consideration before later commerce actions?","definition":"This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","trigger":"Push once after the primary product detail and selected default variant are rendered.","locations":[{"page_type":"product_detail","url_pattern":"https://example.com/products/{product}","component":"Product detail"}],"parameters":[{"name":"currency","data_layer_path":"ecommerce.currency","classification":"official","scope":"event","type":"string","requirement":"conditional","condition":"Required when value is sent.","definition":"Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","value_rule":"Use the ISO 4217 currency code.","allowed_values":["EUR"],"value_evidence_refs":["currencies"],"example":"EUR","source":"Commerce currency configuration.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"exact","checked_date":"2026-08-01","official_text":"Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately."},"value_mode":"technical_identifier"},{"name":"value","data_layer_path":"ecommerce.value","classification":"official","scope":"event","type":"number","requirement":"optional","definition":"Monetary value of the event’s items, excluding shipping and tax.","value_rule":"Set value to the sum of price * quantity for all items; exclude shipping and tax.","example":129.9,"source":"Selected product offer.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"faithful_adaptation","checked_date":"2026-08-01","official_text":"The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value."},"value_mode":"numeric","value_evidence_refs":["item_values"]},{"name":"items","data_layer_path":"ecommerce.items","classification":"official","scope":"event","type":"array","requirement":"required","definition":"The items for the event.","value_rule":"Send one item object for the displayed product variant.","example":[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white","price":129.9,"quantity":1}],"source":"Selected product and variant data.","destination":"ga4_event_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item parameters","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The items for the event."},"value_mode":"structured","value_evidence_refs":["item_arrays"]},{"name":"item_id","data_layer_path":"ecommerce.items[].item_id","classification":"official","scope":"item","type":"string","requirement":"required","definition":"The ID of the item. *One of item_id or item_name is required.","value_rule":"Use the stable SKU or product identifier.","example":"SKU-123","source":"Product catalog.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The ID of the item. *One of item_id or item_name is required."},"value_mode":"technical_identifier","value_evidence_refs":["item_ids"]},{"name":"item_name","data_layer_path":"ecommerce.items[].item_name","classification":"official","scope":"item","type":"string","requirement":"required","definition":"The name of the item. *One of item_id or item_name is required.","value_rule":"Use the stable catalog product name.","example":"Example window","source":"Product catalog.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The name of the item. *One of item_id or item_name is required."},"value_mode":"authoritative_raw","value_evidence_refs":["item_names"]},{"name":"item_variant","data_layer_path":"ecommerce.items[].item_variant","classification":"official","scope":"item","type":"string","requirement":"optional","definition":"The item variant or unique code or description for additional item details/options.","value_rule":"Use the primary normalized size or variant representation.","example":"120x100","source":"Selected variant.","destination":"ga4_item_parameter","official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"items parameter","wording_origin":"exact","checked_date":"2026-08-01","official_text":"The item variant or unique code or description for additional item details/options."},"value_mode":"authoritative_raw","value_evidence_refs":["item_variants"]},{"name":"item_color","data_layer_path":"ecommerce.items[].item_color","classification":"custom","scope":"item","type":"string","requirement":"optional","definition":"Identifies the normalized color selected for the item.","value_rule":"Use the normalized catalog color label.","allowed_values":["white","black","oak"],"value_evidence_refs":["item_colors"],"example":"white","source":"Selected variant color.","destination":"ga4_item_parameter","custom_decision":{"business_need":"Analyse color preference independently from size.","official_candidate":"item_variant","why_not_fit":"item_variant represents the primary size or variant; it cannot isolate color when both dimensions are selected."},"value_mode":"controlled_semantic","value_language":"en"},{"destination":"ga4_item_parameter","value_rule":"Use the selected offer unit price excluding tax and shipping. This fictional supplied offer has no discount.","definition":"The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.","example":129.9,"requirement":"required","name":"price","value_evidence_refs":["item_price"],"data_layer_path":"ecommerce.items[].price","source":"Supplied selected-product offer specification.","official_source":{"official_text":"The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.","wording_origin":"exact","url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"Item parameters","checked_date":"2026-09-27"},"type":"number","classification":"official","value_mode":"numeric","scope":"item"},{"destination":"ga4_item_parameter","value_rule":"Use 1 for the single displayed product unit.","definition":"Item quantity. If not set, quantity is set to 1.","example":1,"requirement":"required","name":"quantity","value_evidence_refs":["item_quantity"],"data_layer_path":"ecommerce.items[].quantity","source":"Supplied selected-product offer specification.","official_source":{"official_text":"Item quantity. If not set, quantity is set to 1.","wording_origin":"exact","url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"Item parameters","checked_date":"2026-09-27"},"type":"number","classification":"official","value_mode":"numeric","scope":"item"}],"data_layer":{"clear":["ecommerce"],"push":{"event":"view_item","ecommerce":{"currency":"EUR","value":129.9,"items":[{"item_id":"SKU-123","item_name":"Example window","item_variant":"120x100","item_color":"white","price":129.9,"quantity":1}]}}},"official_source":{"url":"https://developers.google.com/analytics/devguides/collection/ga4/reference/events#view_item","section":"view_item","wording_origin":"exact","checked_date":"2026-08-01","official_text":"This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed."}},{"event_name":"begin_quote","classification":"custom","journey_ids":["quote_request"],"business_question":"How many visitors intentionally enter the quote journey, and for which project types?","definition":"Indicates that a visitor intentionally started the quote-request journey.","trigger":"Push once when the visitor enters the first interactive quote step after selecting a quote call to action.","locations":[{"page_type":"quote_form","url_pattern":"https://example.com/request-a-quote","component":"Quote form"}],"parameters":[{"name":"form_name","data_layer_path":"event_data.form_name","classification":"custom","scope":"event","type":"string","requirement":"required","definition":"Identifies the form whose journey was started.","value_rule":"Use the stable functional form name.","allowed_values":["quote_request"],"value_evidence_refs":["form_names"],"example":"quote_request","source":"Form configuration.","destination":"ga4_event_parameter","custom_decision":{"business_need":"Compare quote starts for reusable form implementations.","official_candidate":"No prescribed begin_quote parameter identifies the form.","why_not_fit":"A stable form identifier is required to analyse multiple quote entry points."},"value_mode":"controlled_semantic","value_language":"en"},{"name":"project_type","data_layer_path":"event_data.project_type","classification":"custom","scope":"event","type":"string","requirement":"conditional","condition":"Send when the project type is known at journey start.","definition":"Identifies the normalized project selected for the quote request.","value_rule":"Use one of the exhaustive website project types.","allowed_values":["window","door","shutter"],"value_evidence_refs":["project_types"],"example":"window","source":"Selected project option.","destination":"ga4_event_parameter","custom_decision":{"business_need":"Analyse quote starts by requested project.","official_candidate":"No official begin_quote parameter represents the requested project.","why_not_fit":"The project is a business-specific quote dimension."},"value_mode":"controlled_semantic","value_language":"en"}],"data_layer":{"clear":["event_data"],"push":{"event":"begin_quote","event_data":{"form_name":"quote_request","project_type":"window"}}},"custom_decision":{"business_need":"Measure intentional entry into a quote journey before a lead exists.","official_candidate":"form_start","why_not_fit":"The business requires a quote-specific funnel start across interfaces that do not all expose a standard form start."}}]}</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2751,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"projection_version":"1.0.0","sheets":[{"title":"Guide","state":"visible","cells":[["A1","Example GA4 tracking plan","s",null],["A2","Human contract for analyst review, maintenance, and dataLayer implementation.","s",null],["A4","Document","s",null],["B4","Example GA4 tracking plan","s",null],["A5","Version","s",null],["B5","1.0","s",null],["A6","Date","s",null],["B6","2026-08-01","s",null],["A7","Scope","s",null],["B7","Product discovery and quote request","s",null],["A8","Target state","s",null],["B8","to_be","s",null],["A9","Language","s",null],["B9","en","s",null],["A10","Analyst entry point","s",null],["B10","Review journeys and events in Event Matrix.","s","#'Event Matrix'!A1"],["A11","Developer entry point","s",null],["B11","Open an event tab for the exact dataLayer specification.","s","#'core_data'!A1"],["A12","dataLayer convention","s",null],["B12","Default web dataLayer (default)\nClear event_data or ecommerce before replacing a previously populated object.","s",null],["A14","Journeys","s",null],["A15","Journey","s",null],["B15","Scope","s",null],["C15","Business goal","s",null],["D15","URLs / routes","s",null],["A16","Product discovery","s",null],["B16","Product detail pages","s",null],["C16","Understand qualified product interest.","s",null],["D16","https://example.com/products/{product}","s",null],["A17","Quote request","s",null],["B17","Quote form","s",null],["C17","Measure intentional quote starts and accepted leads.","s",null],["D17","https://example.com/request-a-quote","s",null]],"merged_cells":["A14:G14","A1:G1","A2:G2","B10:G10","B11:G11","B12:G12","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"Event Matrix","state":"visible","cells":[["A1","Event Matrix","s",null],["A2","One row per manually implemented event or context push.","s",null],["A4","Event","s",null],["B4","Definition","s",null],["A5","core_data","s","#'core_data'!A1"],["B5","Provides the reusable page and user context needed by subsequent measurement.","s",null],["A6","view_item","s","#'view_item'!A1"],["B6","This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","s",null],["A7","begin_quote","s","#'begin_quote'!A1"],["B7","Indicates that a visitor intentionally started the quote-request journey.","s",null]],"merged_cells":["A1:B1","A2:B2"]},{"title":"Parameter Reference","state":"visible","cells":[["A1","Parameter Reference","s",null],["A2","Definitions and values for parameters actually used by the event specifications.","s",null],["A4","Variable","s",null],["B4","Scope","s",null],["C4","Type","s",null],["D4","Definition","s",null],["E4","Rule","s",null],["F4","Possible values or examples","s",null],["A5","currency","s",null],["B5","event","s",null],["C5","string","s",null],["D5","Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","s",null],["E5","Use the ISO 4217 currency code.","s",null],["F5","EUR","s",null],["A6","form_name","s",null],["B6","event","s",null],["C6","string","s",null],["D6","Identifies the form whose journey was started.","s",null],["E6","Use the stable functional form name.","s",null],["F6","quote_request","s",null],["A7","item_color","s",null],["B7","item","s",null],["C7","string","s",null],["D7","Identifies the normalized color selected for the item.","s",null],["E7","Use the normalized catalog color label.","s",null],["F7","white | black | oak","s",null],["A8","item_id","s",null],["B8","item","s",null],["C8","string","s",null],["D8","The ID of the item. *One of item_id or item_name is required.","s",null],["E8","Use the stable SKU or product identifier.","s",null],["F8","SKU-123","s",null],["A9","item_name","s",null],["B9","item","s",null],["C9","string","s",null],["D9","The name of the item. *One of item_id or item_name is required.","s",null],["E9","Use the stable catalog product name.","s",null],["F9","Example window","s",null],["A10","item_variant","s",null],["B10","item","s",null],["C10","string","s",null],["D10","The item variant or unique code or description for additional item details/options.","s",null],["E10","Use the primary normalized size or variant representation.","s",null],["F10","120x100","s",null],["A11","items","s",null],["B11","event","s",null],["C11","array","s",null],["D11","The items for the event.","s",null],["E11","Send one item object for the displayed product variant.","s",null],["F11","[{\"item_id\":\"SKU-123\",\"item_name\":\"Example window\",\"item_variant\":\"120x100\",\"item_color\":\"white\"}]","s",null],["A12","login_status","s",null],["B12","user","s",null],["C12","string","s",null],["D12","Indicates whether the current visitor is authenticated.","s",null],["E12","Use one of the exhaustive normalized states.","s",null],["F12","logged_out | logged_in","s",null],["A13","page_template","s",null],["B13","implementation","s",null],["C13","string","s",null],["D13","Identifies the stable functional template of the displayed page or route.","s",null],["E13","Use the normalized functional page template.","s",null],["F13","home | product_detail | quote_form | confirmation","s",null],["A14","project_type","s",null],["B14","event","s",null],["C14","string","s",null],["D14","Identifies the normalized project selected for the quote request.","s",null],["E14","Use one of the exhaustive website project types.","s",null],["F14","window | door | shutter","s",null],["A15","user_id","s",null],["B15","user","s",null],["C15","string","s",null],["D15","Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","s",null],["E15","Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.","s",null],["F15","customer_12345","s",null],["A16","value","s",null],["B16","event","s",null],["C16","number","s",null],["D16","The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value.","s",null],["E16","Set value to the sum of price * quantity for all items; exclude shipping and tax.","s",null],["F16","129.9","s",null]],"merged_cells":["A1:F1","A2:F2"]},{"title":"core_data","state":"visible","cells":[["A1","Event: \"core_data\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","core_data","s",null],["A4","Classification","s",null],["B4","dataLayer context","s",null],["A5","Journey","s",null],["B5","Product discovery | Quote request","s",null],["A6","Definition","s",null],["B6","Provides the reusable page and user context needed by subsequent measurement.","s",null],["A7","Trigger","s",null],["B7","Push on every full page load and SPA route change after page and user state are available, and refresh the same context after an authentication-state change.","s",null],["A8","Pages / routes / components","s",null],["B8","all_pages | https://example.com/*","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","page_template","s",null],["B12","implementation","s",null],["C12","string","s",null],["D12","mandatory","s",null],["E12","Identifies the stable functional template of the displayed page or route.","s",null],["F12","Use the normalized functional page template.","s",null],["G12","home | product_detail | quote_form | confirmation","s",null],["A13","login_status","s",null],["B13","user","s",null],["C13","string","s",null],["D13","mandatory","s",null],["E13","Indicates whether the current visitor is authenticated.","s",null],["F13","Use one of the exhaustive normalized states.","s",null],["G13","logged_out | logged_in","s",null],["A14","user_id","s",null],["B14","user","s",null],["C14","string","s",null],["D14","conditional","s",null],["E14","Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","s",null],["F14","Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.","s",null],["G14","customer_12345","s",null],["A16","dataLayer specification","s",null],["A17","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\n  \"page\": {\n    \"page_template\": \"product_detail\"\n  },\n  \"user\": {\n    \"login_status\": \"logged_in\",\n    \"user_id\": \"customer_12345\"\n  }\n});","s",null]],"merged_cells":["A16:G16","A17:G17","A1:G1","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"view_item","state":"visible","cells":[["A1","Event: \"view_item\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","view_item","s",null],["A4","Classification","s",null],["B4","official ecommerce","s",null],["A5","Journey","s",null],["B5","Product discovery","s",null],["A6","Definition","s",null],["B6","This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","s",null],["A7","Trigger","s",null],["B7","Push once after the primary product detail and selected default variant are rendered.","s",null],["A8","Pages / routes / components","s",null],["B8","product_detail | https://example.com/products/{product} | Product detail","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","currency","s",null],["B12","event","s",null],["C12","string","s",null],["D12","conditional","s",null],["E12","Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","s",null],["F12","Use the ISO 4217 currency code.","s",null],["G12","EUR","s",null],["A13","value","s",null],["B13","event","s",null],["C13","number","s",null],["D13","optional","s",null],["E13","The monetary value of the event. * Set value to the sum of (price * quantity) for all items in items. Don't include shipping or tax. * value is typically required for meaningful reporting. If you mark the event as a key event then it's recommended you set value. * currency is required if you set value.","s",null],["F13","Set value to the sum of price * quantity for all items; exclude shipping and tax.","s",null],["G13","129.9","s",null],["A14","items","s",null],["B14","event","s",null],["C14","array","s",null],["D14","mandatory","s",null],["E14","The items for the event.","s",null],["F14","Send one item object for the displayed product variant.","s",null],["G14","[{\"item_id\":\"SKU-123\",\"item_name\":\"Example window\",\"item_variant\":\"120x100\",\"item_color\":\"white\"}]","s",null],["A15","item_id","s",null],["B15","item","s",null],["C15","string","s",null],["D15","mandatory","s",null],["E15","The ID of the item. *One of item_id or item_name is required.","s",null],["F15","Use the stable SKU or product identifier.","s",null],["G15","SKU-123","s",null],["A16","item_name","s",null],["B16","item","s",null],["C16","string","s",null],["D16","mandatory","s",null],["E16","The name of the item. *One of item_id or item_name is required.","s",null],["F16","Use the stable catalog product name.","s",null],["G16","Example window","s",null],["A17","item_variant","s",null],["B17","item","s",null],["C17","string","s",null],["D17","optional","s",null],["E17","The item variant or unique code or description for additional item details/options.","s",null],["F17","Use the primary normalized size or variant representation.","s",null],["G17","120x100","s",null],["A18","item_color","s",null],["B18","item","s",null],["C18","string","s",null],["D18","optional","s",null],["E18","Identifies the normalized color selected for the item.","s",null],["F18","Use the normalized catalog color label.","s",null],["G18","white | black | oak","s",null],["A20","dataLayer specification","s",null],["A21","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\"ecommerce\": null});\nwindow.dataLayer.push({\n  \"event\": \"view_item\",\n  \"ecommerce\": {\n    \"currency\": \"EUR\",\n    \"value\": 129.9,\n    \"items\": [\n      {\n        \"item_id\": \"SKU-123\",\n        \"item_name\": \"Example window\",\n        \"item_variant\": \"120x100\",\n        \"item_color\": \"white\"\n      }\n    ]\n  }\n});","s",null]],"merged_cells":["A1:G1","A20:G20","A21:G21","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"begin_quote","state":"visible","cells":[["A1","Event: \"begin_quote\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","begin_quote","s",null],["A4","Classification","s",null],["B4","custom","s",null],["A5","Journey","s",null],["B5","Quote request","s",null],["A6","Definition","s",null],["B6","Indicates that a visitor intentionally started the quote-request journey.","s",null],["A7","Trigger","s",null],["B7","Push once when the visitor enters the first interactive quote step after selecting a quote call to action.","s",null],["A8","Pages / routes / components","s",null],["B8","quote_form | https://example.com/request-a-quote | Quote form","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","form_name","s",null],["B12","event","s",null],["C12","string","s",null],["D12","mandatory","s",null],["E12","Identifies the form whose journey was started.","s",null],["F12","Use the stable functional form name.","s",null],["G12","quote_request","s",null],["A13","project_type","s",null],["B13","event","s",null],["C13","string","s",null],["D13","conditional","s",null],["E13","Identifies the normalized project selected for the quote request.","s",null],["F13","Use one of the exhaustive website project types.","s",null],["G13","window | door | shutter","s",null],["A15","dataLayer specification","s",null],["A16","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\"event_data\": null});\nwindow.dataLayer.push({\n  \"event\": \"begin_quote\",\n  \"event_data\": {\n    \"form_name\": \"quote_request\",\n    \"project_type\": \"window\"\n  }\n});","s",null]],"merged_cells":["A15:G15","A16:G16","A1:G1","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]}]}</t>
+          <t>{"projection_version":"1.0.0","sheets":[{"title":"Guide","state":"visible","cells":[["A1","Example GA4 tracking plan","s",null],["A2","Human contract for analyst review, maintenance, and dataLayer implementation.","s",null],["A3","Approved — current-source checks passed","s",null],["A4","Document","s",null],["B4","Example GA4 tracking plan","s",null],["A5","Version","s",null],["B5","1.0","s",null],["A6","Date","s",null],["B6","2026-08-01","s",null],["A7","Scope","s",null],["B7","Product discovery and quote request","s",null],["A8","Target state","s",null],["B8","to_be","s",null],["A9","Language","s",null],["B9","en","s",null],["A10","Analyst entry point","s",null],["B10","Review journeys and events in Event Matrix.","s","#'Event Matrix'!A1"],["A11","Developer entry point","s",null],["B11","Open an event tab for the exact dataLayer specification.","s","#'core_data'!A1"],["A12","dataLayer convention","s",null],["B12","Default web dataLayer (default)\nClear event_data or ecommerce before replacing a previously populated object.","s",null],["A14","Journeys","s",null],["A15","Journey","s",null],["B15","Scope","s",null],["C15","Business goal","s",null],["D15","URLs / routes","s",null],["A16","Product discovery","s",null],["B16","Product detail pages","s",null],["C16","Understand qualified product interest.","s",null],["D16","https://example.com/products/{product}","s",null],["A17","Quote request","s",null],["B17","Quote form","s",null],["C17","Measure intentional quote starts and accepted leads.","s",null],["D17","https://example.com/request-a-quote","s",null]],"merged_cells":["A14:G14","A1:G1","A2:G2","A3:G3","B10:G10","B11:G11","B12:G12","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"Event Matrix","state":"visible","cells":[["A1","Event Matrix","s",null],["A2","One row per manually implemented event or context push.","s",null],["A4","Event","s",null],["B4","Definition","s",null],["A5","core_data","s","#'core_data'!A1"],["B5","Provides the reusable page and user context needed by subsequent measurement.","s",null],["A6","view_item","s","#'view_item'!A1"],["B6","This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","s",null],["A7","begin_quote","s","#'begin_quote'!A1"],["B7","Indicates that a visitor intentionally started the quote-request journey.","s",null]],"merged_cells":["A1:B1","A2:B2"]},{"title":"Parameter Reference","state":"visible","cells":[["A1","Parameter Reference","s",null],["A2","Definitions and values for parameters actually used by the event specifications.","s",null],["A4","Variable","s",null],["B4","Scope","s",null],["C4","Type","s",null],["D4","Definition","s",null],["E4","Rule","s",null],["F4","Possible values or examples","s",null],["A5","currency","s",null],["B5","event","s",null],["C5","string","s",null],["D5","Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","s",null],["E5","Use the ISO 4217 currency code.","s",null],["F5","EUR","s",null],["A6","form_name","s",null],["B6","event","s",null],["C6","string","s",null],["D6","Identifies the form whose journey was started.","s",null],["E6","Use the stable functional form name.","s",null],["F6","quote_request","s",null],["A7","item_color","s",null],["B7","item","s",null],["C7","string","s",null],["D7","Identifies the normalized color selected for the item.","s",null],["E7","Use the normalized catalog color label.","s",null],["F7","white | black | oak","s",null],["A8","item_id","s",null],["B8","item","s",null],["C8","string","s",null],["D8","The ID of the item. *One of item_id or item_name is required.","s",null],["E8","Use the stable SKU or product identifier.","s",null],["F8","Example: SKU-123","s",null],["A9","item_name","s",null],["B9","item","s",null],["C9","string","s",null],["D9","The name of the item. *One of item_id or item_name is required.","s",null],["E9","Use the stable catalog product name.","s",null],["F9","Example: Example window","s",null],["A10","item_variant","s",null],["B10","item","s",null],["C10","string","s",null],["D10","The item variant or unique code or description for additional item details/options.","s",null],["E10","Use the primary normalized size or variant representation.","s",null],["F10","Example: 120x100","s",null],["A11","items","s",null],["B11","event","s",null],["C11","array","s",null],["D11","The items for the event.","s",null],["E11","Send one item object for the displayed product variant.","s",null],["F11","See event-specific specifications: view_item","s",null],["A12","login_status","s",null],["B12","user","s",null],["C12","string","s",null],["D12","Indicates whether the current visitor is authenticated.","s",null],["E12","Use one of the exhaustive normalized states.","s",null],["F12","logged_out | logged_in","s",null],["A13","page_template","s",null],["B13","implementation","s",null],["C13","string","s",null],["D13","Identifies the stable functional template of the displayed page or route.","s",null],["E13","Use the normalized functional page template.","s",null],["F13","home | product_detail | quote_form | confirmation","s",null],["A14","price","s",null],["B14","item","s",null],["C14","number","s",null],["D14","The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.","s",null],["E14","Use the selected offer unit price excluding tax and shipping. This fictional supplied offer has no discount.","s",null],["F14","Example: 129.9","s",null],["A15","project_type","s",null],["B15","event","s",null],["C15","string","s",null],["D15","Identifies the normalized project selected for the quote request.","s",null],["E15","Use one of the exhaustive website project types.","s",null],["F15","window | door | shutter","s",null],["A16","quantity","s",null],["B16","item","s",null],["C16","number","s",null],["D16","Item quantity. If not set, quantity is set to 1.","s",null],["E16","Use 1 for the single displayed product unit.","s",null],["F16","Example: 1","s",null],["A17","user_id","s",null],["B17","user","s",null],["C17","string or null","s",null],["D17","Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","s",null],["E17","Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.","s",null],["F17","Example: customer_12345","s",null],["A18","value","s",null],["B18","event","s",null],["C18","number","s",null],["D18","Monetary value of the event’s items, excluding shipping and tax.","s",null],["E18","Set value to the sum of price * quantity for all items; exclude shipping and tax.","s",null],["F18","Example: 129.9","s",null]],"merged_cells":["A1:F1","A2:F2"]},{"title":"core_data","state":"visible","cells":[["A1","Event: \"core_data\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","core_data","s",null],["A4","Classification","s",null],["B4","dataLayer context","s",null],["A5","Journey","s",null],["B5","Product discovery | Quote request","s",null],["A6","Definition","s",null],["B6","Provides the reusable page and user context needed by subsequent measurement.","s",null],["A7","Trigger","s",null],["B7","Push on every full page load and SPA route change after page and user state are available, and refresh the same context after an authentication-state change.","s",null],["A8","Pages / routes / components","s",null],["B8","all_pages | https://example.com/*","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","page_template","s",null],["B12","implementation","s",null],["C12","string","s",null],["D12","mandatory","s",null],["E12","Identifies the stable functional template of the displayed page or route.","s",null],["F12","Use the normalized functional page template.","s",null],["G12","home | product_detail | quote_form | confirmation","s",null],["A13","login_status","s",null],["B13","user","s",null],["C13","string","s",null],["D13","mandatory","s",null],["E13","Indicates whether the current visitor is authenticated.","s",null],["F13","Use one of the exhaustive normalized states.","s",null],["G13","logged_out | logged_in","s",null],["A14","user_id","s",null],["B14","user","s",null],["C14","string or null","s",null],["D14","conditional","s",null],["E14","Identifies the stable first-party account identifier mapped to the official GA4 User-ID configuration setting.","s",null],["F14","Use the stable opaque account identifier; never use an email address or register the value as a custom dimension.\nCondition: Omit user_id before the first sign-in. Send the stable opaque account identifier as a string while signed in. After sign-out, send user_id as null to clear the GA4 User-ID setting.","s",null],["G14","customer_12345","s",null],["A16","dataLayer specification","s",null],["A17","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\n  \"page\": {\n    \"page_template\": \"product_detail\"\n  },\n  \"user\": {\n    \"login_status\": \"logged_in\",\n    \"user_id\": \"customer_12345\"\n  }\n});","s",null]],"merged_cells":["A16:G16","A17:G17","A1:G1","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"view_item","state":"visible","cells":[["A1","Event: \"view_item\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","view_item","s",null],["A4","Classification","s",null],["B4","official ecommerce","s",null],["A5","Journey","s",null],["B5","Product discovery","s",null],["A6","Definition","s",null],["B6","This event signifies that some content was shown to the user. Use this event to discover the most popular items viewed.","s",null],["A7","Trigger","s",null],["B7","Push once after the primary product detail and selected default variant are rendered.","s",null],["A8","Pages / routes / components","s",null],["B8","product_detail | https://example.com/products/{product} | Product detail","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","currency","s",null],["B12","event","s",null],["C12","string","s",null],["D12","conditional","s",null],["E12","Currency of the items associated with the event, in 3-letter ISO 4217 format. * Value metrics on the view_item event to not contribute to revenue * If you set value then currency is required for revenue metrics to be computed accurately.","s",null],["F12","Use the ISO 4217 currency code.\nCondition: Required when value is sent.","s",null],["G12","EUR","s",null],["A13","value","s",null],["B13","event","s",null],["C13","number","s",null],["D13","optional","s",null],["E13","Monetary value of the event’s items, excluding shipping and tax.","s",null],["F13","Set value to the sum of price * quantity for all items; exclude shipping and tax.","s",null],["G13","129.9","s",null],["A14","items","s",null],["B14","event","s",null],["C14","array","s",null],["D14","mandatory","s",null],["E14","The items for the event.","s",null],["F14","Send one item object for the displayed product variant.","s",null],["G14","See the complete dataLayer example.","s",null],["A15","item_id","s",null],["B15","item","s",null],["C15","string","s",null],["D15","mandatory","s",null],["E15","The ID of the item. *One of item_id or item_name is required.","s",null],["F15","Use the stable SKU or product identifier.","s",null],["G15","SKU-123","s",null],["A16","item_name","s",null],["B16","item","s",null],["C16","string","s",null],["D16","mandatory","s",null],["E16","The name of the item. *One of item_id or item_name is required.","s",null],["F16","Use the stable catalog product name.","s",null],["G16","Example window","s",null],["A17","item_variant","s",null],["B17","item","s",null],["C17","string","s",null],["D17","optional","s",null],["E17","The item variant or unique code or description for additional item details/options.","s",null],["F17","Use the primary normalized size or variant representation.","s",null],["G17","120x100","s",null],["A18","item_color","s",null],["B18","item","s",null],["C18","string","s",null],["D18","optional","s",null],["E18","Identifies the normalized color selected for the item.","s",null],["F18","Use the normalized catalog color label.","s",null],["G18","white | black | oak","s",null],["A19","price","s",null],["B19","item","s",null],["C19","number","s",null],["D19","mandatory","s",null],["E19","The monetary unit price of the item, in units of the specified currency parameter. If a discount applies to the item, set price to the discounted unit price and specify the unit price discount in the discount parameter.","s",null],["F19","Use the selected offer unit price excluding tax and shipping. This fictional supplied offer has no discount.","s",null],["G19","129.9","s",null],["A20","quantity","s",null],["B20","item","s",null],["C20","number","s",null],["D20","mandatory","s",null],["E20","Item quantity. If not set, quantity is set to 1.","s",null],["F20","Use 1 for the single displayed product unit.","s",null],["G20","1","s",null],["A22","dataLayer specification","s",null],["A23","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\"ecommerce\": null});\nwindow.dataLayer.push({\n  \"event\": \"view_item\",\n  \"ecommerce\": {\n    \"currency\": \"EUR\",\n    \"value\": 129.9,\n    \"items\": [\n      {\n        \"item_id\": \"SKU-123\",\n        \"item_name\": \"Example window\",\n        \"item_variant\": \"120x100\",\n        \"item_color\": \"white\",\n        \"price\": 129.9,\n        \"quantity\": 1\n      }\n    ]\n  }\n});","s",null]],"merged_cells":["A1:G1","A22:G22","A23:G23","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]},{"title":"begin_quote","state":"visible","cells":[["A1","Event: \"begin_quote\"","s",null],["A2","Authoritative event, parameter, and dataLayer specification.","s",null],["A3","Event","s",null],["B3","begin_quote","s",null],["A4","Classification","s",null],["B4","custom","s",null],["A5","Journey","s",null],["B5","Quote request","s",null],["A6","Definition","s",null],["B6","Indicates that a visitor intentionally started the quote-request journey.","s",null],["A7","Trigger","s",null],["B7","Push once when the visitor enters the first interactive quote step after selecting a quote call to action.","s",null],["A8","Pages / routes / components","s",null],["B8","quote_form | https://example.com/request-a-quote | Quote form","s",null],["A9","Notes","s",null],["A11","Variable","s",null],["B11","Scope","s",null],["C11","Type","s",null],["D11","Requirement","s",null],["E11","Definition","s",null],["F11","Rule","s",null],["G11","Possible values or examples","s",null],["A12","form_name","s",null],["B12","event","s",null],["C12","string","s",null],["D12","mandatory","s",null],["E12","Identifies the form whose journey was started.","s",null],["F12","Use the stable functional form name.","s",null],["G12","quote_request","s",null],["A13","project_type","s",null],["B13","event","s",null],["C13","string","s",null],["D13","conditional","s",null],["E13","Identifies the normalized project selected for the quote request.","s",null],["F13","Use one of the exhaustive website project types.\nCondition: Send when the project type is known at journey start.","s",null],["G13","window | door | shutter","s",null],["A15","dataLayer specification","s",null],["A16","window.dataLayer = window.dataLayer || [];\nwindow.dataLayer.push({\"event_data\": null});\nwindow.dataLayer.push({\n  \"event\": \"begin_quote\",\n  \"event_data\": {\n    \"form_name\": \"quote_request\",\n    \"project_type\": \"window\"\n  }\n});","s",null]],"merged_cells":["A15:G15","A16:G16","A1:G1","A2:G2","B3:G3","B4:G4","B5:G5","B6:G6","B7:G7","B8:G8","B9:G9"]}]}</t>
         </is>
       </c>
     </row>

</xml_diff>